<commit_message>
ibkr's grants were calculated worng due splits
</commit_message>
<xml_diff>
--- a/data/aix_pref.xlsx
+++ b/data/aix_pref.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I1286"/>
+  <dimension ref="A1:I1315"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -53148,6 +53148,1253 @@
         </is>
       </c>
     </row>
+    <row r="1287">
+      <c r="A1287" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="B1287" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="C1287" t="inlineStr">
+        <is>
+          <t>AIRA</t>
+        </is>
+      </c>
+      <c r="D1287" t="inlineStr">
+        <is>
+          <t>Ordinary Shares of Air Astana JSC</t>
+        </is>
+      </c>
+      <c r="E1287" t="inlineStr">
+        <is>
+          <t>AIR ASTANA JSC</t>
+        </is>
+      </c>
+      <c r="F1287" t="inlineStr">
+        <is>
+          <t>EQTY</t>
+        </is>
+      </c>
+      <c r="G1287" t="n">
+        <v>1293</v>
+      </c>
+      <c r="H1287" t="n">
+        <v>81613659.11</v>
+      </c>
+      <c r="I1287" t="inlineStr">
+        <is>
+          <t>KZ1C00004050</t>
+        </is>
+      </c>
+    </row>
+    <row r="1288">
+      <c r="A1288" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="B1288" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="C1288" t="inlineStr">
+        <is>
+          <t>AIRA.U</t>
+        </is>
+      </c>
+      <c r="D1288" t="inlineStr">
+        <is>
+          <t>Ordinary Shares of Air Astana JSC</t>
+        </is>
+      </c>
+      <c r="E1288" t="inlineStr">
+        <is>
+          <t>AIR ASTANA JSC</t>
+        </is>
+      </c>
+      <c r="F1288" t="inlineStr">
+        <is>
+          <t>EQTY</t>
+        </is>
+      </c>
+      <c r="G1288" t="n">
+        <v>873</v>
+      </c>
+      <c r="H1288" t="n">
+        <v>88506680.8</v>
+      </c>
+      <c r="I1288" t="inlineStr">
+        <is>
+          <t>KZ1CCCCCCCC3</t>
+        </is>
+      </c>
+    </row>
+    <row r="1289">
+      <c r="A1289" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="B1289" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="C1289" t="inlineStr">
+        <is>
+          <t>AIRA.Y</t>
+        </is>
+      </c>
+      <c r="D1289" t="inlineStr">
+        <is>
+          <t>GDRs of Air Astana JSC</t>
+        </is>
+      </c>
+      <c r="E1289" t="inlineStr">
+        <is>
+          <t>AIR ASTANA JSC</t>
+        </is>
+      </c>
+      <c r="F1289" t="inlineStr">
+        <is>
+          <t>EQTY</t>
+        </is>
+      </c>
+      <c r="G1289" t="n">
+        <v>197</v>
+      </c>
+      <c r="H1289" t="n">
+        <v>1038552643.28</v>
+      </c>
+      <c r="I1289" t="inlineStr">
+        <is>
+          <t>US0090632078</t>
+        </is>
+      </c>
+    </row>
+    <row r="1290">
+      <c r="A1290" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="B1290" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="C1290" t="inlineStr">
+        <is>
+          <t>ALMS</t>
+        </is>
+      </c>
+      <c r="D1290" t="inlineStr">
+        <is>
+          <t>Ordinary Shares of ALMS</t>
+        </is>
+      </c>
+      <c r="E1290" t="inlineStr">
+        <is>
+          <t>AK Altynalmas JSC</t>
+        </is>
+      </c>
+      <c r="F1290" t="inlineStr">
+        <is>
+          <t>EQTY</t>
+        </is>
+      </c>
+      <c r="G1290" t="n">
+        <v>0</v>
+      </c>
+      <c r="H1290" t="n">
+        <v>0</v>
+      </c>
+      <c r="I1290" t="inlineStr">
+        <is>
+          <t>KZ1C00001080</t>
+        </is>
+      </c>
+    </row>
+    <row r="1291">
+      <c r="A1291" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="B1291" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="C1291" t="inlineStr">
+        <is>
+          <t>ALMSP</t>
+        </is>
+      </c>
+      <c r="D1291" t="inlineStr">
+        <is>
+          <t>Preferred Shares of ALMS</t>
+        </is>
+      </c>
+      <c r="E1291" t="inlineStr">
+        <is>
+          <t>AK Altynalmas JSC</t>
+        </is>
+      </c>
+      <c r="F1291" t="inlineStr">
+        <is>
+          <t>EQTY</t>
+        </is>
+      </c>
+      <c r="G1291" t="n">
+        <v>0</v>
+      </c>
+      <c r="H1291" t="n">
+        <v>0</v>
+      </c>
+      <c r="I1291" t="inlineStr">
+        <is>
+          <t>KZ1P00001093</t>
+        </is>
+      </c>
+    </row>
+    <row r="1292">
+      <c r="A1292" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="B1292" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="C1292" t="inlineStr">
+        <is>
+          <t>CCBN</t>
+        </is>
+      </c>
+      <c r="D1292" t="inlineStr">
+        <is>
+          <t>Ordinary Shares of JSC Bank CenterCredit</t>
+        </is>
+      </c>
+      <c r="E1292" t="inlineStr">
+        <is>
+          <t>JSC Bank CenterCredit</t>
+        </is>
+      </c>
+      <c r="F1292" t="inlineStr">
+        <is>
+          <t>EQTY</t>
+        </is>
+      </c>
+      <c r="G1292" t="n">
+        <v>373</v>
+      </c>
+      <c r="H1292" t="n">
+        <v>125166389.08</v>
+      </c>
+      <c r="I1292" t="inlineStr">
+        <is>
+          <t>KZ0007786572</t>
+        </is>
+      </c>
+    </row>
+    <row r="1293">
+      <c r="A1293" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="B1293" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="C1293" t="inlineStr">
+        <is>
+          <t>CORE</t>
+        </is>
+      </c>
+      <c r="D1293" t="inlineStr">
+        <is>
+          <t>Ordinary Shares of Solidcore Resources</t>
+        </is>
+      </c>
+      <c r="E1293" t="inlineStr">
+        <is>
+          <t>SOLIDCORE RESOURCES PLC</t>
+        </is>
+      </c>
+      <c r="F1293" t="inlineStr">
+        <is>
+          <t>EQTY</t>
+        </is>
+      </c>
+      <c r="G1293" t="n">
+        <v>4771</v>
+      </c>
+      <c r="H1293" t="n">
+        <v>7204526698.09</v>
+      </c>
+      <c r="I1293" t="inlineStr">
+        <is>
+          <t>JE00B6T5S470</t>
+        </is>
+      </c>
+    </row>
+    <row r="1294">
+      <c r="A1294" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="B1294" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="C1294" t="inlineStr">
+        <is>
+          <t>CORE.K</t>
+        </is>
+      </c>
+      <c r="D1294" t="inlineStr">
+        <is>
+          <t>Ordinary Shares of Solidcore Resources KZT</t>
+        </is>
+      </c>
+      <c r="E1294" t="inlineStr">
+        <is>
+          <t>SOLIDCORE RESOURCES PLC</t>
+        </is>
+      </c>
+      <c r="F1294" t="inlineStr">
+        <is>
+          <t>EQTY</t>
+        </is>
+      </c>
+      <c r="G1294" t="n">
+        <v>260</v>
+      </c>
+      <c r="H1294" t="n">
+        <v>76741826.56999999</v>
+      </c>
+      <c r="I1294" t="inlineStr">
+        <is>
+          <t>KZAAAAAAAAA5</t>
+        </is>
+      </c>
+    </row>
+    <row r="1295">
+      <c r="A1295" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="B1295" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="C1295" t="inlineStr">
+        <is>
+          <t>EUA</t>
+        </is>
+      </c>
+      <c r="D1295" t="inlineStr">
+        <is>
+          <t>Ordinary Shares of Eurasia Mining PLC</t>
+        </is>
+      </c>
+      <c r="E1295" t="inlineStr">
+        <is>
+          <t>Eurasia Mining PLC</t>
+        </is>
+      </c>
+      <c r="F1295" t="inlineStr">
+        <is>
+          <t>EQTY</t>
+        </is>
+      </c>
+      <c r="G1295" t="n">
+        <v>61</v>
+      </c>
+      <c r="H1295" t="n">
+        <v>855835.41</v>
+      </c>
+      <c r="I1295" t="inlineStr">
+        <is>
+          <t>GB0003230421</t>
+        </is>
+      </c>
+    </row>
+    <row r="1296">
+      <c r="A1296" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="B1296" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="C1296" t="inlineStr">
+        <is>
+          <t>FAR</t>
+        </is>
+      </c>
+      <c r="D1296" t="inlineStr">
+        <is>
+          <t>Ordinary shares of Ferro-Alloy Recources LTD</t>
+        </is>
+      </c>
+      <c r="E1296" t="inlineStr">
+        <is>
+          <t>Ferro-Alloy Resources Limited</t>
+        </is>
+      </c>
+      <c r="F1296" t="inlineStr">
+        <is>
+          <t>EQTY</t>
+        </is>
+      </c>
+      <c r="G1296" t="n">
+        <v>84</v>
+      </c>
+      <c r="H1296" t="n">
+        <v>9345775.119999999</v>
+      </c>
+      <c r="I1296" t="inlineStr">
+        <is>
+          <t>GG00BGDYDZ69</t>
+        </is>
+      </c>
+    </row>
+    <row r="1297">
+      <c r="A1297" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="B1297" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="C1297" t="inlineStr">
+        <is>
+          <t>FIXP.Y</t>
+        </is>
+      </c>
+      <c r="D1297" t="inlineStr">
+        <is>
+          <t>GDRs of Fix Price Group PLC</t>
+        </is>
+      </c>
+      <c r="E1297" t="inlineStr">
+        <is>
+          <t>FIX PRICE GROUP PLC</t>
+        </is>
+      </c>
+      <c r="F1297" t="inlineStr">
+        <is>
+          <t>EQTY</t>
+        </is>
+      </c>
+      <c r="G1297" t="n">
+        <v>50</v>
+      </c>
+      <c r="H1297" t="n">
+        <v>7573333.87</v>
+      </c>
+      <c r="I1297" t="inlineStr">
+        <is>
+          <t>US33835G2057</t>
+        </is>
+      </c>
+    </row>
+    <row r="1298">
+      <c r="A1298" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="B1298" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="C1298" t="inlineStr">
+        <is>
+          <t>FRHC</t>
+        </is>
+      </c>
+      <c r="D1298" t="inlineStr">
+        <is>
+          <t>Ordinary shares of Freedom Holding Corp.</t>
+        </is>
+      </c>
+      <c r="E1298" t="inlineStr">
+        <is>
+          <t>Freedom Holding Corp</t>
+        </is>
+      </c>
+      <c r="F1298" t="inlineStr">
+        <is>
+          <t>EQTY</t>
+        </is>
+      </c>
+      <c r="G1298" t="n">
+        <v>11</v>
+      </c>
+      <c r="H1298" t="n">
+        <v>55690460.39</v>
+      </c>
+      <c r="I1298" t="inlineStr">
+        <is>
+          <t>US3563901046</t>
+        </is>
+      </c>
+    </row>
+    <row r="1299">
+      <c r="A1299" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="B1299" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="C1299" t="inlineStr">
+        <is>
+          <t>HSBK</t>
+        </is>
+      </c>
+      <c r="D1299" t="inlineStr">
+        <is>
+          <t>Common Shares of JSC Halyk Savings Bank of Kazakhstan</t>
+        </is>
+      </c>
+      <c r="E1299" t="inlineStr">
+        <is>
+          <t>Joint Stock Company "Halyk Bank of Kazakhstan"</t>
+        </is>
+      </c>
+      <c r="F1299" t="inlineStr">
+        <is>
+          <t>EQTY</t>
+        </is>
+      </c>
+      <c r="G1299" t="n">
+        <v>3113</v>
+      </c>
+      <c r="H1299" t="n">
+        <v>60103134.77</v>
+      </c>
+      <c r="I1299" t="inlineStr">
+        <is>
+          <t>KZ000A0LE0S4</t>
+        </is>
+      </c>
+    </row>
+    <row r="1300">
+      <c r="A1300" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="B1300" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="C1300" t="inlineStr">
+        <is>
+          <t>HSBK.Y</t>
+        </is>
+      </c>
+      <c r="D1300" t="inlineStr">
+        <is>
+          <t>GDRs of "Halyk Savings Bank of Kazakhstan" JSC</t>
+        </is>
+      </c>
+      <c r="E1300" t="inlineStr">
+        <is>
+          <t>Joint Stock Company "Halyk Bank of Kazakhstan"</t>
+        </is>
+      </c>
+      <c r="F1300" t="inlineStr">
+        <is>
+          <t>EQTY</t>
+        </is>
+      </c>
+      <c r="G1300" t="n">
+        <v>136</v>
+      </c>
+      <c r="H1300" t="n">
+        <v>67596527.98</v>
+      </c>
+      <c r="I1300" t="inlineStr">
+        <is>
+          <t>US46627J3023</t>
+        </is>
+      </c>
+    </row>
+    <row r="1301">
+      <c r="A1301" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="B1301" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="C1301" t="inlineStr">
+        <is>
+          <t>JXIR</t>
+        </is>
+      </c>
+      <c r="D1301" t="inlineStr">
+        <is>
+          <t>Ordinary Shares of Jiaxin International</t>
+        </is>
+      </c>
+      <c r="E1301" t="inlineStr">
+        <is>
+          <t>JIAXIN INTERNATIONAL RESOURCES INVESTMENT Ltd</t>
+        </is>
+      </c>
+      <c r="F1301" t="inlineStr">
+        <is>
+          <t>EQTY</t>
+        </is>
+      </c>
+      <c r="G1301" t="n">
+        <v>207</v>
+      </c>
+      <c r="H1301" t="n">
+        <v>25948442.55</v>
+      </c>
+      <c r="I1301" t="inlineStr">
+        <is>
+          <t>HK0001188587</t>
+        </is>
+      </c>
+    </row>
+    <row r="1302">
+      <c r="A1302" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="B1302" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="C1302" t="inlineStr">
+        <is>
+          <t>KAP</t>
+        </is>
+      </c>
+      <c r="D1302" t="inlineStr">
+        <is>
+          <t>Ordinary Shares of NC "Kazatomprom" JSC</t>
+        </is>
+      </c>
+      <c r="E1302" t="inlineStr">
+        <is>
+          <t>Joint Stock Company National Atomic Company "Kazatomprom"</t>
+        </is>
+      </c>
+      <c r="F1302" t="inlineStr">
+        <is>
+          <t>EQTY</t>
+        </is>
+      </c>
+      <c r="G1302" t="n">
+        <v>497</v>
+      </c>
+      <c r="H1302" t="n">
+        <v>176215284.02</v>
+      </c>
+      <c r="I1302" t="inlineStr">
+        <is>
+          <t>KZ1C00001619</t>
+        </is>
+      </c>
+    </row>
+    <row r="1303">
+      <c r="A1303" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="B1303" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="C1303" t="inlineStr">
+        <is>
+          <t>KAP.Y</t>
+        </is>
+      </c>
+      <c r="D1303" t="inlineStr">
+        <is>
+          <t>Global Depository Receipts of NC "Kazatomprom" JSC</t>
+        </is>
+      </c>
+      <c r="E1303" t="inlineStr">
+        <is>
+          <t>Joint Stock Company National Atomic Company "Kazatomprom"</t>
+        </is>
+      </c>
+      <c r="F1303" t="inlineStr">
+        <is>
+          <t>EQTY</t>
+        </is>
+      </c>
+      <c r="G1303" t="n">
+        <v>107</v>
+      </c>
+      <c r="H1303" t="n">
+        <v>41624082.14</v>
+      </c>
+      <c r="I1303" t="inlineStr">
+        <is>
+          <t>US63253R2013</t>
+        </is>
+      </c>
+    </row>
+    <row r="1304">
+      <c r="A1304" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="B1304" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="C1304" t="inlineStr">
+        <is>
+          <t>KEGC</t>
+        </is>
+      </c>
+      <c r="D1304" t="inlineStr">
+        <is>
+          <t>Ordinary Shares of KEGOC JSC</t>
+        </is>
+      </c>
+      <c r="E1304" t="inlineStr">
+        <is>
+          <t>KEGOC JSC</t>
+        </is>
+      </c>
+      <c r="F1304" t="inlineStr">
+        <is>
+          <t>EQTY</t>
+        </is>
+      </c>
+      <c r="G1304" t="n">
+        <v>832</v>
+      </c>
+      <c r="H1304" t="n">
+        <v>20152523.76</v>
+      </c>
+      <c r="I1304" t="inlineStr">
+        <is>
+          <t>KZ1C00000959</t>
+        </is>
+      </c>
+    </row>
+    <row r="1305">
+      <c r="A1305" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="B1305" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="C1305" t="inlineStr">
+        <is>
+          <t>KMG</t>
+        </is>
+      </c>
+      <c r="D1305" t="inlineStr">
+        <is>
+          <t>Ordinary Shares of NC "KazMunayGas" JSC</t>
+        </is>
+      </c>
+      <c r="E1305" t="inlineStr">
+        <is>
+          <t>JSC NC KazMunayGas</t>
+        </is>
+      </c>
+      <c r="F1305" t="inlineStr">
+        <is>
+          <t>EQTY</t>
+        </is>
+      </c>
+      <c r="G1305" t="n">
+        <v>313</v>
+      </c>
+      <c r="H1305" t="n">
+        <v>190982779.04</v>
+      </c>
+      <c r="I1305" t="inlineStr">
+        <is>
+          <t>KZ1C00001122</t>
+        </is>
+      </c>
+    </row>
+    <row r="1306">
+      <c r="A1306" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="B1306" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="C1306" t="inlineStr">
+        <is>
+          <t>KSPI</t>
+        </is>
+      </c>
+      <c r="D1306" t="inlineStr">
+        <is>
+          <t>AMERICAN DEPOSITORY SHARES OF JSC "KASPI.KZ"</t>
+        </is>
+      </c>
+      <c r="E1306" t="inlineStr">
+        <is>
+          <t>JOINT STOCK COMPANY "KASPI.KZ"</t>
+        </is>
+      </c>
+      <c r="F1306" t="inlineStr">
+        <is>
+          <t>EQTY</t>
+        </is>
+      </c>
+      <c r="G1306" t="n">
+        <v>119</v>
+      </c>
+      <c r="H1306" t="n">
+        <v>93130948.28</v>
+      </c>
+      <c r="I1306" t="inlineStr">
+        <is>
+          <t>US48581R2058</t>
+        </is>
+      </c>
+    </row>
+    <row r="1307">
+      <c r="A1307" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="B1307" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="C1307" t="inlineStr">
+        <is>
+          <t>KSPI.S</t>
+        </is>
+      </c>
+      <c r="D1307" t="inlineStr">
+        <is>
+          <t>COMMON SHARES OF JSC KASPI.KZ</t>
+        </is>
+      </c>
+      <c r="E1307" t="inlineStr">
+        <is>
+          <t>JOINT STOCK COMPANY "KASPI.KZ"</t>
+        </is>
+      </c>
+      <c r="F1307" t="inlineStr">
+        <is>
+          <t>EQTY</t>
+        </is>
+      </c>
+      <c r="G1307" t="n">
+        <v>0</v>
+      </c>
+      <c r="H1307" t="n">
+        <v>0</v>
+      </c>
+      <c r="I1307" t="inlineStr">
+        <is>
+          <t>KZ1C00001536</t>
+        </is>
+      </c>
+    </row>
+    <row r="1308">
+      <c r="A1308" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="B1308" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="C1308" t="inlineStr">
+        <is>
+          <t>KZHY010625AK</t>
+        </is>
+      </c>
+      <c r="D1308" t="inlineStr">
+        <is>
+          <t>I-RECs of 2.5 MW Turkestan HPP</t>
+        </is>
+      </c>
+      <c r="E1308" t="inlineStr">
+        <is>
+          <t>Evident Ev Limited</t>
+        </is>
+      </c>
+      <c r="F1308" t="inlineStr">
+        <is>
+          <t>EQTY</t>
+        </is>
+      </c>
+      <c r="G1308" t="n">
+        <v>0</v>
+      </c>
+      <c r="H1308" t="n">
+        <v>0</v>
+      </c>
+      <c r="I1308" t="inlineStr">
+        <is>
+          <t>KZZ111111118</t>
+        </is>
+      </c>
+    </row>
+    <row r="1309">
+      <c r="A1309" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="B1309" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="C1309" t="inlineStr">
+        <is>
+          <t>KZSO080924S2</t>
+        </is>
+      </c>
+      <c r="D1309" t="inlineStr">
+        <is>
+          <t>I-RECs of SPP 2MW SGE</t>
+        </is>
+      </c>
+      <c r="E1309" t="inlineStr">
+        <is>
+          <t>Evident Ev Limited</t>
+        </is>
+      </c>
+      <c r="F1309" t="inlineStr">
+        <is>
+          <t>EQTY</t>
+        </is>
+      </c>
+      <c r="G1309" t="n">
+        <v>0</v>
+      </c>
+      <c r="H1309" t="n">
+        <v>0</v>
+      </c>
+      <c r="I1309" t="inlineStr">
+        <is>
+          <t>KZ1666666667</t>
+        </is>
+      </c>
+    </row>
+    <row r="1310">
+      <c r="A1310" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="B1310" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="C1310" t="inlineStr">
+        <is>
+          <t>KZSO101224S2</t>
+        </is>
+      </c>
+      <c r="D1310" t="inlineStr">
+        <is>
+          <t>I-RECs of SPP 2MW SGE</t>
+        </is>
+      </c>
+      <c r="E1310" t="inlineStr">
+        <is>
+          <t>Evident Ev Limited</t>
+        </is>
+      </c>
+      <c r="F1310" t="inlineStr">
+        <is>
+          <t>EQTY</t>
+        </is>
+      </c>
+      <c r="G1310" t="n">
+        <v>0</v>
+      </c>
+      <c r="H1310" t="n">
+        <v>0</v>
+      </c>
+      <c r="I1310" t="inlineStr">
+        <is>
+          <t>KZ1666666659</t>
+        </is>
+      </c>
+    </row>
+    <row r="1311">
+      <c r="A1311" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="B1311" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="C1311" t="inlineStr">
+        <is>
+          <t>KZWI020225ES</t>
+        </is>
+      </c>
+      <c r="D1311" t="inlineStr">
+        <is>
+          <t>I-RECs of 60 MW WPP Shelek</t>
+        </is>
+      </c>
+      <c r="E1311" t="inlineStr">
+        <is>
+          <t>Evident Ev Limited</t>
+        </is>
+      </c>
+      <c r="F1311" t="inlineStr">
+        <is>
+          <t>EQTY</t>
+        </is>
+      </c>
+      <c r="G1311" t="n">
+        <v>0</v>
+      </c>
+      <c r="H1311" t="n">
+        <v>0</v>
+      </c>
+      <c r="I1311" t="inlineStr">
+        <is>
+          <t>KZ1666666550</t>
+        </is>
+      </c>
+    </row>
+    <row r="1312">
+      <c r="A1312" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="B1312" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="C1312" t="inlineStr">
+        <is>
+          <t>NNDQ</t>
+        </is>
+      </c>
+      <c r="D1312" t="inlineStr">
+        <is>
+          <t>American Depositary Shares of Nanduq PLC</t>
+        </is>
+      </c>
+      <c r="E1312" t="inlineStr">
+        <is>
+          <t>NanduQ PLC</t>
+        </is>
+      </c>
+      <c r="F1312" t="inlineStr">
+        <is>
+          <t>EQTY</t>
+        </is>
+      </c>
+      <c r="G1312" t="n">
+        <v>1</v>
+      </c>
+      <c r="H1312" t="n">
+        <v>1324.42</v>
+      </c>
+      <c r="I1312" t="inlineStr">
+        <is>
+          <t>US74735M1080</t>
+        </is>
+      </c>
+    </row>
+    <row r="1313">
+      <c r="A1313" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="B1313" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="C1313" t="inlineStr">
+        <is>
+          <t>SOG</t>
+        </is>
+      </c>
+      <c r="D1313" t="inlineStr">
+        <is>
+          <t>Ordinary shares of "Sozak Oil and Gas" Joint Stock Company</t>
+        </is>
+      </c>
+      <c r="E1313" t="inlineStr">
+        <is>
+          <t>SOZAK OIL AND GAS JSC</t>
+        </is>
+      </c>
+      <c r="F1313" t="inlineStr">
+        <is>
+          <t>EQTY</t>
+        </is>
+      </c>
+      <c r="G1313" t="n">
+        <v>0</v>
+      </c>
+      <c r="H1313" t="n">
+        <v>0</v>
+      </c>
+      <c r="I1313" t="inlineStr">
+        <is>
+          <t>KZ1C00013630</t>
+        </is>
+      </c>
+    </row>
+    <row r="1314">
+      <c r="A1314" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="B1314" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="C1314" t="inlineStr">
+        <is>
+          <t>TCIB</t>
+        </is>
+      </c>
+      <c r="D1314" t="inlineStr">
+        <is>
+          <t>Shares of Teniz Capital Investment Banking</t>
+        </is>
+      </c>
+      <c r="E1314" t="inlineStr">
+        <is>
+          <t>Teniz Capital Invetsment Banking JSC</t>
+        </is>
+      </c>
+      <c r="F1314" t="inlineStr">
+        <is>
+          <t>EQTY</t>
+        </is>
+      </c>
+      <c r="G1314" t="n">
+        <v>31</v>
+      </c>
+      <c r="H1314" t="n">
+        <v>110416553</v>
+      </c>
+      <c r="I1314" t="inlineStr">
+        <is>
+          <t>KZ1C00000256</t>
+        </is>
+      </c>
+    </row>
+    <row r="1315">
+      <c r="A1315" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="B1315" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="C1315" t="inlineStr">
+        <is>
+          <t>UZHY010125CH</t>
+        </is>
+      </c>
+      <c r="D1315" t="inlineStr">
+        <is>
+          <t>I-RECs of 666 MW Charvak HPP</t>
+        </is>
+      </c>
+      <c r="E1315" t="inlineStr">
+        <is>
+          <t>Evident Ev Limited</t>
+        </is>
+      </c>
+      <c r="F1315" t="inlineStr">
+        <is>
+          <t>EQTY</t>
+        </is>
+      </c>
+      <c r="G1315" t="n">
+        <v>0</v>
+      </c>
+      <c r="H1315" t="n">
+        <v>0</v>
+      </c>
+      <c r="I1315" t="inlineStr">
+        <is>
+          <t>SBRFEEQXBR28</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
audit file list order has changed
</commit_message>
<xml_diff>
--- a/data/aix_pref.xlsx
+++ b/data/aix_pref.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I1315"/>
+  <dimension ref="A1:I1344"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -54395,6 +54395,1253 @@
         </is>
       </c>
     </row>
+    <row r="1316">
+      <c r="A1316" t="inlineStr">
+        <is>
+          <t>2026-08</t>
+        </is>
+      </c>
+      <c r="B1316" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="C1316" t="inlineStr">
+        <is>
+          <t>ALMS</t>
+        </is>
+      </c>
+      <c r="D1316" t="inlineStr">
+        <is>
+          <t>Ordinary Shares of ALMS</t>
+        </is>
+      </c>
+      <c r="E1316" t="inlineStr">
+        <is>
+          <t>AK Altynalmas JSC</t>
+        </is>
+      </c>
+      <c r="F1316" t="inlineStr">
+        <is>
+          <t>EQTY</t>
+        </is>
+      </c>
+      <c r="G1316" t="n">
+        <v>0</v>
+      </c>
+      <c r="H1316" t="n">
+        <v>0</v>
+      </c>
+      <c r="I1316" t="inlineStr">
+        <is>
+          <t>KZ1C00001080</t>
+        </is>
+      </c>
+    </row>
+    <row r="1317">
+      <c r="A1317" t="inlineStr">
+        <is>
+          <t>2026-08</t>
+        </is>
+      </c>
+      <c r="B1317" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="C1317" t="inlineStr">
+        <is>
+          <t>ALMSP</t>
+        </is>
+      </c>
+      <c r="D1317" t="inlineStr">
+        <is>
+          <t>Preferred Shares of ALMS</t>
+        </is>
+      </c>
+      <c r="E1317" t="inlineStr">
+        <is>
+          <t>AK Altynalmas JSC</t>
+        </is>
+      </c>
+      <c r="F1317" t="inlineStr">
+        <is>
+          <t>EQTY</t>
+        </is>
+      </c>
+      <c r="G1317" t="n">
+        <v>0</v>
+      </c>
+      <c r="H1317" t="n">
+        <v>0</v>
+      </c>
+      <c r="I1317" t="inlineStr">
+        <is>
+          <t>KZ1P00001093</t>
+        </is>
+      </c>
+    </row>
+    <row r="1318">
+      <c r="A1318" t="inlineStr">
+        <is>
+          <t>2026-08</t>
+        </is>
+      </c>
+      <c r="B1318" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="C1318" t="inlineStr">
+        <is>
+          <t>KSPI.S</t>
+        </is>
+      </c>
+      <c r="D1318" t="inlineStr">
+        <is>
+          <t>COMMON SHARES OF JSC KASPI.KZ</t>
+        </is>
+      </c>
+      <c r="E1318" t="inlineStr">
+        <is>
+          <t>JOINT STOCK COMPANY "KASPI.KZ"</t>
+        </is>
+      </c>
+      <c r="F1318" t="inlineStr">
+        <is>
+          <t>EQTY</t>
+        </is>
+      </c>
+      <c r="G1318" t="n">
+        <v>0</v>
+      </c>
+      <c r="H1318" t="n">
+        <v>0</v>
+      </c>
+      <c r="I1318" t="inlineStr">
+        <is>
+          <t>KZ1C00001536</t>
+        </is>
+      </c>
+    </row>
+    <row r="1319">
+      <c r="A1319" t="inlineStr">
+        <is>
+          <t>2026-08</t>
+        </is>
+      </c>
+      <c r="B1319" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="C1319" t="inlineStr">
+        <is>
+          <t>KZHY010625AK</t>
+        </is>
+      </c>
+      <c r="D1319" t="inlineStr">
+        <is>
+          <t>I-RECs of 2.5 MW Turkestan HPP</t>
+        </is>
+      </c>
+      <c r="E1319" t="inlineStr">
+        <is>
+          <t>Evident Ev Limited</t>
+        </is>
+      </c>
+      <c r="F1319" t="inlineStr">
+        <is>
+          <t>EQTY</t>
+        </is>
+      </c>
+      <c r="G1319" t="n">
+        <v>0</v>
+      </c>
+      <c r="H1319" t="n">
+        <v>0</v>
+      </c>
+      <c r="I1319" t="inlineStr">
+        <is>
+          <t>KZZ111111118</t>
+        </is>
+      </c>
+    </row>
+    <row r="1320">
+      <c r="A1320" t="inlineStr">
+        <is>
+          <t>2026-08</t>
+        </is>
+      </c>
+      <c r="B1320" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="C1320" t="inlineStr">
+        <is>
+          <t>KZSO080924S2</t>
+        </is>
+      </c>
+      <c r="D1320" t="inlineStr">
+        <is>
+          <t>I-RECs of SPP 2MW SGE</t>
+        </is>
+      </c>
+      <c r="E1320" t="inlineStr">
+        <is>
+          <t>Evident Ev Limited</t>
+        </is>
+      </c>
+      <c r="F1320" t="inlineStr">
+        <is>
+          <t>EQTY</t>
+        </is>
+      </c>
+      <c r="G1320" t="n">
+        <v>0</v>
+      </c>
+      <c r="H1320" t="n">
+        <v>0</v>
+      </c>
+      <c r="I1320" t="inlineStr">
+        <is>
+          <t>KZ1666666667</t>
+        </is>
+      </c>
+    </row>
+    <row r="1321">
+      <c r="A1321" t="inlineStr">
+        <is>
+          <t>2026-08</t>
+        </is>
+      </c>
+      <c r="B1321" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="C1321" t="inlineStr">
+        <is>
+          <t>KZSO101224S2</t>
+        </is>
+      </c>
+      <c r="D1321" t="inlineStr">
+        <is>
+          <t>I-RECs of SPP 2MW SGE</t>
+        </is>
+      </c>
+      <c r="E1321" t="inlineStr">
+        <is>
+          <t>Evident Ev Limited</t>
+        </is>
+      </c>
+      <c r="F1321" t="inlineStr">
+        <is>
+          <t>EQTY</t>
+        </is>
+      </c>
+      <c r="G1321" t="n">
+        <v>0</v>
+      </c>
+      <c r="H1321" t="n">
+        <v>0</v>
+      </c>
+      <c r="I1321" t="inlineStr">
+        <is>
+          <t>KZ1666666659</t>
+        </is>
+      </c>
+    </row>
+    <row r="1322">
+      <c r="A1322" t="inlineStr">
+        <is>
+          <t>2026-08</t>
+        </is>
+      </c>
+      <c r="B1322" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="C1322" t="inlineStr">
+        <is>
+          <t>KZWI020225ES</t>
+        </is>
+      </c>
+      <c r="D1322" t="inlineStr">
+        <is>
+          <t>I-RECs of 60 MW WPP Shelek</t>
+        </is>
+      </c>
+      <c r="E1322" t="inlineStr">
+        <is>
+          <t>Evident Ev Limited</t>
+        </is>
+      </c>
+      <c r="F1322" t="inlineStr">
+        <is>
+          <t>EQTY</t>
+        </is>
+      </c>
+      <c r="G1322" t="n">
+        <v>0</v>
+      </c>
+      <c r="H1322" t="n">
+        <v>0</v>
+      </c>
+      <c r="I1322" t="inlineStr">
+        <is>
+          <t>KZ1666666550</t>
+        </is>
+      </c>
+    </row>
+    <row r="1323">
+      <c r="A1323" t="inlineStr">
+        <is>
+          <t>2026-08</t>
+        </is>
+      </c>
+      <c r="B1323" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="C1323" t="inlineStr">
+        <is>
+          <t>SOG</t>
+        </is>
+      </c>
+      <c r="D1323" t="inlineStr">
+        <is>
+          <t>Ordinary shares of "Sozak Oil and Gas" Joint Stock Company</t>
+        </is>
+      </c>
+      <c r="E1323" t="inlineStr">
+        <is>
+          <t>SOZAK OIL AND GAS JSC</t>
+        </is>
+      </c>
+      <c r="F1323" t="inlineStr">
+        <is>
+          <t>EQTY</t>
+        </is>
+      </c>
+      <c r="G1323" t="n">
+        <v>0</v>
+      </c>
+      <c r="H1323" t="n">
+        <v>0</v>
+      </c>
+      <c r="I1323" t="inlineStr">
+        <is>
+          <t>KZ1C00013630</t>
+        </is>
+      </c>
+    </row>
+    <row r="1324">
+      <c r="A1324" t="inlineStr">
+        <is>
+          <t>2026-08</t>
+        </is>
+      </c>
+      <c r="B1324" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="C1324" t="inlineStr">
+        <is>
+          <t>UZHY010125CH</t>
+        </is>
+      </c>
+      <c r="D1324" t="inlineStr">
+        <is>
+          <t>I-RECs of 666 MW Charvak HPP</t>
+        </is>
+      </c>
+      <c r="E1324" t="inlineStr">
+        <is>
+          <t>Evident Ev Limited</t>
+        </is>
+      </c>
+      <c r="F1324" t="inlineStr">
+        <is>
+          <t>EQTY</t>
+        </is>
+      </c>
+      <c r="G1324" t="n">
+        <v>0</v>
+      </c>
+      <c r="H1324" t="n">
+        <v>0</v>
+      </c>
+      <c r="I1324" t="inlineStr">
+        <is>
+          <t>SBRFEEQXBR28</t>
+        </is>
+      </c>
+    </row>
+    <row r="1325">
+      <c r="A1325" t="inlineStr">
+        <is>
+          <t>2026-08</t>
+        </is>
+      </c>
+      <c r="B1325" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="C1325" t="inlineStr">
+        <is>
+          <t>TCIB</t>
+        </is>
+      </c>
+      <c r="D1325" t="inlineStr">
+        <is>
+          <t>Shares of Teniz Capital Investment Banking</t>
+        </is>
+      </c>
+      <c r="E1325" t="inlineStr">
+        <is>
+          <t>Teniz Capital Invetsment Banking JSC</t>
+        </is>
+      </c>
+      <c r="F1325" t="inlineStr">
+        <is>
+          <t>EQTY</t>
+        </is>
+      </c>
+      <c r="G1325" t="n">
+        <v>15</v>
+      </c>
+      <c r="H1325" t="n">
+        <v>45992934</v>
+      </c>
+      <c r="I1325" t="inlineStr">
+        <is>
+          <t>KZ1C00000256</t>
+        </is>
+      </c>
+    </row>
+    <row r="1326">
+      <c r="A1326" t="inlineStr">
+        <is>
+          <t>2026-08</t>
+        </is>
+      </c>
+      <c r="B1326" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="C1326" t="inlineStr">
+        <is>
+          <t>NNDQ</t>
+        </is>
+      </c>
+      <c r="D1326" t="inlineStr">
+        <is>
+          <t>American Depositary Shares of Nanduq PLC</t>
+        </is>
+      </c>
+      <c r="E1326" t="inlineStr">
+        <is>
+          <t>NanduQ PLC</t>
+        </is>
+      </c>
+      <c r="F1326" t="inlineStr">
+        <is>
+          <t>EQTY</t>
+        </is>
+      </c>
+      <c r="G1326" t="n">
+        <v>2</v>
+      </c>
+      <c r="H1326" t="n">
+        <v>23705.92</v>
+      </c>
+      <c r="I1326" t="inlineStr">
+        <is>
+          <t>US74735M1080</t>
+        </is>
+      </c>
+    </row>
+    <row r="1327">
+      <c r="A1327" t="inlineStr">
+        <is>
+          <t>2026-08</t>
+        </is>
+      </c>
+      <c r="B1327" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="C1327" t="inlineStr">
+        <is>
+          <t>FRHC</t>
+        </is>
+      </c>
+      <c r="D1327" t="inlineStr">
+        <is>
+          <t>Ordinary shares of Freedom Holding Corp.</t>
+        </is>
+      </c>
+      <c r="E1327" t="inlineStr">
+        <is>
+          <t>Freedom Holding Corp</t>
+        </is>
+      </c>
+      <c r="F1327" t="inlineStr">
+        <is>
+          <t>EQTY</t>
+        </is>
+      </c>
+      <c r="G1327" t="n">
+        <v>3</v>
+      </c>
+      <c r="H1327" t="n">
+        <v>2446669.06</v>
+      </c>
+      <c r="I1327" t="inlineStr">
+        <is>
+          <t>US3563901046</t>
+        </is>
+      </c>
+    </row>
+    <row r="1328">
+      <c r="A1328" t="inlineStr">
+        <is>
+          <t>2026-08</t>
+        </is>
+      </c>
+      <c r="B1328" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="C1328" t="inlineStr">
+        <is>
+          <t>AIRA</t>
+        </is>
+      </c>
+      <c r="D1328" t="inlineStr">
+        <is>
+          <t>Ordinary Shares of Air Astana JSC</t>
+        </is>
+      </c>
+      <c r="E1328" t="inlineStr">
+        <is>
+          <t>AIR ASTANA JSC</t>
+        </is>
+      </c>
+      <c r="F1328" t="inlineStr">
+        <is>
+          <t>EQTY</t>
+        </is>
+      </c>
+      <c r="G1328" t="n">
+        <v>1461</v>
+      </c>
+      <c r="H1328" t="n">
+        <v>64075797.3</v>
+      </c>
+      <c r="I1328" t="inlineStr">
+        <is>
+          <t>KZ1C00004050</t>
+        </is>
+      </c>
+    </row>
+    <row r="1329">
+      <c r="A1329" t="inlineStr">
+        <is>
+          <t>2026-08</t>
+        </is>
+      </c>
+      <c r="B1329" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="C1329" t="inlineStr">
+        <is>
+          <t>AIRA.U</t>
+        </is>
+      </c>
+      <c r="D1329" t="inlineStr">
+        <is>
+          <t>Ordinary Shares of Air Astana JSC</t>
+        </is>
+      </c>
+      <c r="E1329" t="inlineStr">
+        <is>
+          <t>AIR ASTANA JSC</t>
+        </is>
+      </c>
+      <c r="F1329" t="inlineStr">
+        <is>
+          <t>EQTY</t>
+        </is>
+      </c>
+      <c r="G1329" t="n">
+        <v>1171</v>
+      </c>
+      <c r="H1329" t="n">
+        <v>166751985.98</v>
+      </c>
+      <c r="I1329" t="inlineStr">
+        <is>
+          <t>KZ1CCCCCCCC3</t>
+        </is>
+      </c>
+    </row>
+    <row r="1330">
+      <c r="A1330" t="inlineStr">
+        <is>
+          <t>2026-08</t>
+        </is>
+      </c>
+      <c r="B1330" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="C1330" t="inlineStr">
+        <is>
+          <t>AIRA.Y</t>
+        </is>
+      </c>
+      <c r="D1330" t="inlineStr">
+        <is>
+          <t>GDRs of Air Astana JSC</t>
+        </is>
+      </c>
+      <c r="E1330" t="inlineStr">
+        <is>
+          <t>AIR ASTANA JSC</t>
+        </is>
+      </c>
+      <c r="F1330" t="inlineStr">
+        <is>
+          <t>EQTY</t>
+        </is>
+      </c>
+      <c r="G1330" t="n">
+        <v>219</v>
+      </c>
+      <c r="H1330" t="n">
+        <v>956418085.9299999</v>
+      </c>
+      <c r="I1330" t="inlineStr">
+        <is>
+          <t>US0090632078</t>
+        </is>
+      </c>
+    </row>
+    <row r="1331">
+      <c r="A1331" t="inlineStr">
+        <is>
+          <t>2026-08</t>
+        </is>
+      </c>
+      <c r="B1331" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="C1331" t="inlineStr">
+        <is>
+          <t>CCBN</t>
+        </is>
+      </c>
+      <c r="D1331" t="inlineStr">
+        <is>
+          <t>Ordinary Shares of JSC Bank CenterCredit</t>
+        </is>
+      </c>
+      <c r="E1331" t="inlineStr">
+        <is>
+          <t>JSC Bank CenterCredit</t>
+        </is>
+      </c>
+      <c r="F1331" t="inlineStr">
+        <is>
+          <t>EQTY</t>
+        </is>
+      </c>
+      <c r="G1331" t="n">
+        <v>430</v>
+      </c>
+      <c r="H1331" t="n">
+        <v>10799434.16</v>
+      </c>
+      <c r="I1331" t="inlineStr">
+        <is>
+          <t>KZ0007786572</t>
+        </is>
+      </c>
+    </row>
+    <row r="1332">
+      <c r="A1332" t="inlineStr">
+        <is>
+          <t>2026-08</t>
+        </is>
+      </c>
+      <c r="B1332" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="C1332" t="inlineStr">
+        <is>
+          <t>CORE</t>
+        </is>
+      </c>
+      <c r="D1332" t="inlineStr">
+        <is>
+          <t>Ordinary Shares of Solidcore Resources</t>
+        </is>
+      </c>
+      <c r="E1332" t="inlineStr">
+        <is>
+          <t>SOLIDCORE RESOURCES PLC</t>
+        </is>
+      </c>
+      <c r="F1332" t="inlineStr">
+        <is>
+          <t>EQTY</t>
+        </is>
+      </c>
+      <c r="G1332" t="n">
+        <v>6275</v>
+      </c>
+      <c r="H1332" t="n">
+        <v>7384965605.34</v>
+      </c>
+      <c r="I1332" t="inlineStr">
+        <is>
+          <t>JE00B6T5S470</t>
+        </is>
+      </c>
+    </row>
+    <row r="1333">
+      <c r="A1333" t="inlineStr">
+        <is>
+          <t>2026-08</t>
+        </is>
+      </c>
+      <c r="B1333" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="C1333" t="inlineStr">
+        <is>
+          <t>CORE.K</t>
+        </is>
+      </c>
+      <c r="D1333" t="inlineStr">
+        <is>
+          <t>Ordinary Shares of Solidcore Resources KZT</t>
+        </is>
+      </c>
+      <c r="E1333" t="inlineStr">
+        <is>
+          <t>SOLIDCORE RESOURCES PLC</t>
+        </is>
+      </c>
+      <c r="F1333" t="inlineStr">
+        <is>
+          <t>EQTY</t>
+        </is>
+      </c>
+      <c r="G1333" t="n">
+        <v>364</v>
+      </c>
+      <c r="H1333" t="n">
+        <v>102892497.16</v>
+      </c>
+      <c r="I1333" t="inlineStr">
+        <is>
+          <t>KZAAAAAAAAA5</t>
+        </is>
+      </c>
+    </row>
+    <row r="1334">
+      <c r="A1334" t="inlineStr">
+        <is>
+          <t>2026-08</t>
+        </is>
+      </c>
+      <c r="B1334" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="C1334" t="inlineStr">
+        <is>
+          <t>EUA</t>
+        </is>
+      </c>
+      <c r="D1334" t="inlineStr">
+        <is>
+          <t>Ordinary Shares of Eurasia Mining PLC</t>
+        </is>
+      </c>
+      <c r="E1334" t="inlineStr">
+        <is>
+          <t>Eurasia Mining PLC</t>
+        </is>
+      </c>
+      <c r="F1334" t="inlineStr">
+        <is>
+          <t>EQTY</t>
+        </is>
+      </c>
+      <c r="G1334" t="n">
+        <v>56</v>
+      </c>
+      <c r="H1334" t="n">
+        <v>310503.71</v>
+      </c>
+      <c r="I1334" t="inlineStr">
+        <is>
+          <t>GB0003230421</t>
+        </is>
+      </c>
+    </row>
+    <row r="1335">
+      <c r="A1335" t="inlineStr">
+        <is>
+          <t>2026-08</t>
+        </is>
+      </c>
+      <c r="B1335" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="C1335" t="inlineStr">
+        <is>
+          <t>FAR</t>
+        </is>
+      </c>
+      <c r="D1335" t="inlineStr">
+        <is>
+          <t>Ordinary shares of Ferro-Alloy Recources LTD</t>
+        </is>
+      </c>
+      <c r="E1335" t="inlineStr">
+        <is>
+          <t>Ferro-Alloy Resources Limited</t>
+        </is>
+      </c>
+      <c r="F1335" t="inlineStr">
+        <is>
+          <t>EQTY</t>
+        </is>
+      </c>
+      <c r="G1335" t="n">
+        <v>87</v>
+      </c>
+      <c r="H1335" t="n">
+        <v>2887624.82</v>
+      </c>
+      <c r="I1335" t="inlineStr">
+        <is>
+          <t>GG00BGDYDZ69</t>
+        </is>
+      </c>
+    </row>
+    <row r="1336">
+      <c r="A1336" t="inlineStr">
+        <is>
+          <t>2026-08</t>
+        </is>
+      </c>
+      <c r="B1336" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="C1336" t="inlineStr">
+        <is>
+          <t>FIXP.Y</t>
+        </is>
+      </c>
+      <c r="D1336" t="inlineStr">
+        <is>
+          <t>GDRs of Fix Price Group PLC</t>
+        </is>
+      </c>
+      <c r="E1336" t="inlineStr">
+        <is>
+          <t>FIX PRICE GROUP PLC</t>
+        </is>
+      </c>
+      <c r="F1336" t="inlineStr">
+        <is>
+          <t>EQTY</t>
+        </is>
+      </c>
+      <c r="G1336" t="n">
+        <v>51</v>
+      </c>
+      <c r="H1336" t="n">
+        <v>16267676.21</v>
+      </c>
+      <c r="I1336" t="inlineStr">
+        <is>
+          <t>US33835G2057</t>
+        </is>
+      </c>
+    </row>
+    <row r="1337">
+      <c r="A1337" t="inlineStr">
+        <is>
+          <t>2026-08</t>
+        </is>
+      </c>
+      <c r="B1337" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="C1337" t="inlineStr">
+        <is>
+          <t>HSBK</t>
+        </is>
+      </c>
+      <c r="D1337" t="inlineStr">
+        <is>
+          <t>Common Shares of JSC Halyk Savings Bank of Kazakhstan</t>
+        </is>
+      </c>
+      <c r="E1337" t="inlineStr">
+        <is>
+          <t>Joint Stock Company "Halyk Bank of Kazakhstan"</t>
+        </is>
+      </c>
+      <c r="F1337" t="inlineStr">
+        <is>
+          <t>EQTY</t>
+        </is>
+      </c>
+      <c r="G1337" t="n">
+        <v>3870</v>
+      </c>
+      <c r="H1337" t="n">
+        <v>129944581.63</v>
+      </c>
+      <c r="I1337" t="inlineStr">
+        <is>
+          <t>KZ000A0LE0S4</t>
+        </is>
+      </c>
+    </row>
+    <row r="1338">
+      <c r="A1338" t="inlineStr">
+        <is>
+          <t>2026-08</t>
+        </is>
+      </c>
+      <c r="B1338" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="C1338" t="inlineStr">
+        <is>
+          <t>HSBK.Y</t>
+        </is>
+      </c>
+      <c r="D1338" t="inlineStr">
+        <is>
+          <t>GDRs of "Halyk Savings Bank of Kazakhstan" JSC</t>
+        </is>
+      </c>
+      <c r="E1338" t="inlineStr">
+        <is>
+          <t>Joint Stock Company "Halyk Bank of Kazakhstan"</t>
+        </is>
+      </c>
+      <c r="F1338" t="inlineStr">
+        <is>
+          <t>EQTY</t>
+        </is>
+      </c>
+      <c r="G1338" t="n">
+        <v>169</v>
+      </c>
+      <c r="H1338" t="n">
+        <v>175175927.24</v>
+      </c>
+      <c r="I1338" t="inlineStr">
+        <is>
+          <t>US46627J3023</t>
+        </is>
+      </c>
+    </row>
+    <row r="1339">
+      <c r="A1339" t="inlineStr">
+        <is>
+          <t>2026-08</t>
+        </is>
+      </c>
+      <c r="B1339" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="C1339" t="inlineStr">
+        <is>
+          <t>JXIR</t>
+        </is>
+      </c>
+      <c r="D1339" t="inlineStr">
+        <is>
+          <t>Ordinary Shares of Jiaxin International</t>
+        </is>
+      </c>
+      <c r="E1339" t="inlineStr">
+        <is>
+          <t>JIAXIN INTERNATIONAL RESOURCES INVESTMENT Ltd</t>
+        </is>
+      </c>
+      <c r="F1339" t="inlineStr">
+        <is>
+          <t>EQTY</t>
+        </is>
+      </c>
+      <c r="G1339" t="n">
+        <v>169</v>
+      </c>
+      <c r="H1339" t="n">
+        <v>27096424.99</v>
+      </c>
+      <c r="I1339" t="inlineStr">
+        <is>
+          <t>HK0001188587</t>
+        </is>
+      </c>
+    </row>
+    <row r="1340">
+      <c r="A1340" t="inlineStr">
+        <is>
+          <t>2026-08</t>
+        </is>
+      </c>
+      <c r="B1340" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="C1340" t="inlineStr">
+        <is>
+          <t>KAP</t>
+        </is>
+      </c>
+      <c r="D1340" t="inlineStr">
+        <is>
+          <t>Ordinary Shares of NC "Kazatomprom" JSC</t>
+        </is>
+      </c>
+      <c r="E1340" t="inlineStr">
+        <is>
+          <t>Joint Stock Company National Atomic Company "Kazatomprom"</t>
+        </is>
+      </c>
+      <c r="F1340" t="inlineStr">
+        <is>
+          <t>EQTY</t>
+        </is>
+      </c>
+      <c r="G1340" t="n">
+        <v>542</v>
+      </c>
+      <c r="H1340" t="n">
+        <v>216433200</v>
+      </c>
+      <c r="I1340" t="inlineStr">
+        <is>
+          <t>KZ1C00001619</t>
+        </is>
+      </c>
+    </row>
+    <row r="1341">
+      <c r="A1341" t="inlineStr">
+        <is>
+          <t>2026-08</t>
+        </is>
+      </c>
+      <c r="B1341" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="C1341" t="inlineStr">
+        <is>
+          <t>KAP.Y</t>
+        </is>
+      </c>
+      <c r="D1341" t="inlineStr">
+        <is>
+          <t>Global Depository Receipts of NC "Kazatomprom" JSC</t>
+        </is>
+      </c>
+      <c r="E1341" t="inlineStr">
+        <is>
+          <t>Joint Stock Company National Atomic Company "Kazatomprom"</t>
+        </is>
+      </c>
+      <c r="F1341" t="inlineStr">
+        <is>
+          <t>EQTY</t>
+        </is>
+      </c>
+      <c r="G1341" t="n">
+        <v>70</v>
+      </c>
+      <c r="H1341" t="n">
+        <v>8609890.26</v>
+      </c>
+      <c r="I1341" t="inlineStr">
+        <is>
+          <t>US63253R2013</t>
+        </is>
+      </c>
+    </row>
+    <row r="1342">
+      <c r="A1342" t="inlineStr">
+        <is>
+          <t>2026-08</t>
+        </is>
+      </c>
+      <c r="B1342" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="C1342" t="inlineStr">
+        <is>
+          <t>KEGC</t>
+        </is>
+      </c>
+      <c r="D1342" t="inlineStr">
+        <is>
+          <t>Ordinary Shares of KEGOC JSC</t>
+        </is>
+      </c>
+      <c r="E1342" t="inlineStr">
+        <is>
+          <t>KEGOC JSC</t>
+        </is>
+      </c>
+      <c r="F1342" t="inlineStr">
+        <is>
+          <t>EQTY</t>
+        </is>
+      </c>
+      <c r="G1342" t="n">
+        <v>1129</v>
+      </c>
+      <c r="H1342" t="n">
+        <v>117049591.33</v>
+      </c>
+      <c r="I1342" t="inlineStr">
+        <is>
+          <t>KZ1C00000959</t>
+        </is>
+      </c>
+    </row>
+    <row r="1343">
+      <c r="A1343" t="inlineStr">
+        <is>
+          <t>2026-08</t>
+        </is>
+      </c>
+      <c r="B1343" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="C1343" t="inlineStr">
+        <is>
+          <t>KMG</t>
+        </is>
+      </c>
+      <c r="D1343" t="inlineStr">
+        <is>
+          <t>Ordinary Shares of NC "KazMunayGas" JSC</t>
+        </is>
+      </c>
+      <c r="E1343" t="inlineStr">
+        <is>
+          <t>JSC NC KazMunayGas</t>
+        </is>
+      </c>
+      <c r="F1343" t="inlineStr">
+        <is>
+          <t>EQTY</t>
+        </is>
+      </c>
+      <c r="G1343" t="n">
+        <v>305</v>
+      </c>
+      <c r="H1343" t="n">
+        <v>245824067.51</v>
+      </c>
+      <c r="I1343" t="inlineStr">
+        <is>
+          <t>KZ1C00001122</t>
+        </is>
+      </c>
+    </row>
+    <row r="1344">
+      <c r="A1344" t="inlineStr">
+        <is>
+          <t>2026-08</t>
+        </is>
+      </c>
+      <c r="B1344" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="C1344" t="inlineStr">
+        <is>
+          <t>KSPI</t>
+        </is>
+      </c>
+      <c r="D1344" t="inlineStr">
+        <is>
+          <t>AMERICAN DEPOSITORY SHARES OF JSC "KASPI.KZ"</t>
+        </is>
+      </c>
+      <c r="E1344" t="inlineStr">
+        <is>
+          <t>JOINT STOCK COMPANY "KASPI.KZ"</t>
+        </is>
+      </c>
+      <c r="F1344" t="inlineStr">
+        <is>
+          <t>EQTY</t>
+        </is>
+      </c>
+      <c r="G1344" t="n">
+        <v>211</v>
+      </c>
+      <c r="H1344" t="n">
+        <v>138643570.02</v>
+      </c>
+      <c r="I1344" t="inlineStr">
+        <is>
+          <t>US48581R2058</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>